<commit_message>
Planilha: separa diagnóstico do site da ação de abordagem
</commit_message>
<xml_diff>
--- a/prospeccao/prospeccao-rvland.xlsx
+++ b/prospeccao/prospeccao-rvland.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Avisos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leads'!$A$4:$O$70</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Prioridade'!$A$4:$O$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leads'!$A$4:$P$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Prioridade'!$A$4:$P$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Instagram'!$A$4:$I$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -155,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -227,8 +227,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -1750,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1767,7 +1773,8 @@
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="62" customWidth="1" min="15" max="15"/>
+    <col width="58" customWidth="1" min="15" max="15"/>
+    <col width="72" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1780,7 +1787,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por potencial. Site, print, Instagram e e-mail são clicáveis: confira cada avaliação você mesmo.</t>
+          <t>Site, print, Instagram e e-mail são clicáveis. As duas últimas colunas são coisas diferentes: o diagnóstico é o que EU vi no site hoje; 'Como abordar' é o que VOCÊ faz.</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1864,12 @@
       </c>
       <c r="O4" s="10" t="inlineStr">
         <is>
-          <t>Ângulo de abordagem</t>
+          <t>O que vi no site (diagnóstico)</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>Como abordar (o que fazer)</t>
         </is>
       </c>
     </row>
@@ -1919,6 +1931,11 @@
       <c r="O5" s="25" t="inlineStr">
         <is>
           <t>Site de 2013 com botoes bisotados; detailing premium (pacotes de USD 350) = tem caixa; redesign completo + booking</t>
+        </is>
+      </c>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t>SEM IG e SEM e-mail no site. Ache 'Macron Mobile Detailing Columbus' no Google Maps/Facebook, ou use o formulário do próprio site. Gancho: mande a prévia junto de 'seu trabalho é premium, o site está em 2013'. Alvo nº1 da lista.</t>
         </is>
       </c>
     </row>
@@ -1978,6 +1995,11 @@
           <t>Layout anos 2000, logo clipart, fundo de bolhas; 2 unidades familiares; redesign + booking</t>
         </is>
       </c>
+      <c r="P6" s="30" t="inlineStr">
+        <is>
+          <t>SEM canal direto no site. Procure 'Octopus Car Wash' no Maps/Facebook. Gancho: print lado a lado (bolhas e clipart) contra a prévia moderna. 2 unidades familiares = fala com o dono.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="n">
@@ -2035,6 +2057,11 @@
           <t>Template generico ~2010, 1 unidade + loja de conveniencia; redesign completo</t>
         </is>
       </c>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>SEM canal direto no site. Buscar no Maps/Facebook. Gancho: 1 unidade + loja de conveniência; prévia com serviços, preços e horário bem visíveis.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="26" t="n">
@@ -2106,6 +2133,11 @@
           <t>No ar desde 2001, layout 2012, embed YouTube antigo; historia forte pra contar num site novo</t>
         </is>
       </c>
+      <c r="P8" s="30" t="inlineStr">
+        <is>
+          <t>DM no @curbsidemobiledetailing (1.583) ou e-mail info@. Gancho: no ar desde 2001 é história forte que o site atual esconde; prévia destacando os 20+ anos.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="n">
@@ -2171,6 +2203,11 @@
           <t>Hero quebrado (secao em branco, form solto); multi-unidades em Orlando; consertar = venda facil de mostrar</t>
         </is>
       </c>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>CUIDADO: os e-mails são de outras franquias. Ache a unidade de Orlando no Maps. Gancho: o hero da home está QUEBRADO (seção em branco com formulário solto); o print é o argumento mais fácil da lista inteira.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="26" t="n">
@@ -2240,6 +2277,11 @@
       <c r="O10" s="30" t="inlineStr">
         <is>
           <t>Hero quebrado com sobreposicao de logo; frota adesivada (investe em marca); ATENCAO: sede em Doral/Miami</t>
+        </is>
+      </c>
+      <c r="P10" s="30" t="inlineStr">
+        <is>
+          <t>DM no @purrfectgrooming.pet (4.980) ou e-mail contactus@. Gancho: hero quebrado com logo sobreposto; frota adesivada mostra que investem em marca, mas o site não acompanha. Confirme a cidade antes (parece Doral, não Orlando).</t>
         </is>
       </c>
     </row>
@@ -2303,6 +2345,11 @@
           <t>Copyright 2011, template bootstrap velho, form denso; negocio real com 2 telefones</t>
         </is>
       </c>
+      <c r="P11" s="25" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps/Facebook. Gancho: copyright 2011 e formulário denso; prévia com pedido de orçamento em 3 campos.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="26" t="n">
@@ -2366,6 +2413,11 @@
       <c r="O12" s="30" t="inlineStr">
         <is>
           <t>Divi roxo datado ~2015; oficina familiar desde 1979; email do dono (mickey@) exposto no site</t>
+        </is>
+      </c>
+      <c r="P12" s="30" t="inlineStr">
+        <is>
+          <t>E-mail DIRETO DO DONO: mickey@phoenixautoshop.com. Gancho: oficina de família desde 1979 com site Divi roxo de 2015; prévia que respeite a história e mostre agendamento.</t>
         </is>
       </c>
     </row>
@@ -2427,6 +2479,11 @@
       <c r="O13" s="25" t="inlineStr">
         <is>
           <t>Visual datado, video com texto arial; rede local pequena de Phoenix</t>
+        </is>
+      </c>
+      <c r="P13" s="25" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps. Gancho: visual datado com texto em Arial sobre vídeo; rede local pequena de Phoenix.</t>
         </is>
       </c>
     </row>
@@ -2486,6 +2543,11 @@
           <t>Weebly DIY, tipografia generica, fotos reais; dono fez sozinho</t>
         </is>
       </c>
+      <c r="P14" s="30" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps/Facebook. Gancho: Weebly feito pelo próprio dono, ele já sabe que o site é fraco; prévia com galeria das cercas reais.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="n">
@@ -2555,6 +2617,11 @@
       <c r="O15" s="25" t="inlineStr">
         <is>
           <t>Logo 3D anos 2000, botoes de ticket; desde 1967, Carrier dealer = caixa; decisao pode ser lenta</t>
+        </is>
+      </c>
+      <c r="P15" s="25" t="inlineStr">
+        <is>
+          <t>E-mail tom@ ou max@ (parecem os sócios) ou DM @westernhvac (2.281). Gancho: desde 1967 e Carrier dealer, mas logo 3D dos anos 2000. Empresa grande: espere decisão mais lenta.</t>
         </is>
       </c>
     </row>
@@ -2618,6 +2685,11 @@
           <t>Template 2012 com foto de banco de imagem; info@ visivel no header</t>
         </is>
       </c>
+      <c r="P16" s="30" t="inlineStr">
+        <is>
+          <t>E-mail info@sciotolandscaping.com. Gancho: template de 2012 usando FOTO DE BANCO DE IMAGEM; prévia com os jardins reais que eles fizeram.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="21" t="n">
@@ -2683,6 +2755,11 @@
           <t>Logo clipart, WP basico; 49 reviews 4.8 = negocio bom com site fraco</t>
         </is>
       </c>
+      <c r="P17" s="25" t="inlineStr">
+        <is>
+          <t>E-mail straightedgepp@gmail.com (Gmail = negócio pequeno, o dono lê). Gancho: 49 avaliações 4.8 estrelas e o site não mostra isso em lugar nenhum.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="26" t="n">
@@ -2754,6 +2831,11 @@
           <t>Wix DIY com logo duplicado gigante e layout desalinhado; tem booking</t>
         </is>
       </c>
+      <c r="P18" s="30" t="inlineStr">
+        <is>
+          <t>DM no @allcreaturespetgrooming (3.277) ou e-mail info@. Gancho: Wix com logo duplicado gigante e layout desalinhado; print lado a lado resolve a conversa.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="21" t="n">
@@ -2821,6 +2903,11 @@
           <t>Layout ~2015 (Duda), logo simples; padaria artesanal com IG</t>
         </is>
       </c>
+      <c r="P19" s="25" t="inlineStr">
+        <is>
+          <t>DM no @bloombakingco (4.204). SEM e-mail no site. Gancho: padaria artesanal bonita com site sem graça; prévia com as fotos dos produtos que já postam no IG.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="26" t="n">
@@ -2886,6 +2973,11 @@
           <t>GoDaddy DIY, 1 unidade; template razoavel mas generico</t>
         </is>
       </c>
+      <c r="P20" s="30" t="inlineStr">
+        <is>
+          <t>E-mail bluswancarwash@gmail.com. Gancho: GoDaddy DIY genérico; prévia com planos e preços claros.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="21" t="n">
@@ -2951,6 +3043,11 @@
       <c r="O21" s="25" t="inlineStr">
         <is>
           <t>Layout centrado antigo; customerservice@ exposto; negocio estabelecido</t>
+        </is>
+      </c>
+      <c r="P21" s="25" t="inlineStr">
+        <is>
+          <t>E-mail customerservice@alamofencesa.com. Gancho: layout centrado antigo. Extra: o IG tem só 88 seguidores, dá pra oferecer site + presença social.</t>
         </is>
       </c>
     </row>
@@ -3014,6 +3111,11 @@
           <t>WP generico, hero cru; empresa 25+ anos</t>
         </is>
       </c>
+      <c r="P22" s="30" t="inlineStr">
+        <is>
+          <t>E-mail service@ims365hvac.com. Gancho: 25+ anos de experiência num WordPress genérico com hero cru.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="21" t="n">
@@ -3081,6 +3183,11 @@
           <t>Logo anos 90, layout mediano; academia local com programas</t>
         </is>
       </c>
+      <c r="P23" s="25" t="inlineStr">
+        <is>
+          <t>DM no @maworlando (1.049) ou e-mail orlandoadmin@. Gancho: logo dos anos 90; prévia com formulário de aula experimental, que é como academia capta.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="n">
@@ -3148,6 +3255,11 @@
           <t>Squarespace generico, logo clipart, hero fraco; facil mostrar upgrade</t>
         </is>
       </c>
+      <c r="P24" s="30" t="inlineStr">
+        <is>
+          <t>E-mail powerwashproplus@gmail.com. Gancho: Squarespace genérico com logo clipart. O IG tem 7 seguidores: está começando do zero, bom candidato a site + social.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="21" t="n">
@@ -3219,6 +3331,11 @@
           <t>Artista solo desde 1997; site simples escuro; decisao rapida, IG e a vida do tatuador</t>
         </is>
       </c>
+      <c r="P25" s="25" t="inlineStr">
+        <is>
+          <t>DM no @wes_tattoos_columbus (11K seguidores!). Gancho: artista solo desde 1997, decisão rápida e sem comitê; IG forte mas site simples, prévia com galeria destacada.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="n">
@@ -3290,6 +3407,11 @@
           <t>Site ok porem copyright 2016; IG ativo 3.5k; abordagem por relacionamento</t>
         </is>
       </c>
+      <c r="P26" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @bubbledowncarwash.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="21" t="n">
@@ -3355,6 +3477,11 @@
           <t>Site decente mas email no Gmail (DIY vibe); familia</t>
         </is>
       </c>
+      <c r="P27" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: e-mail do site.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="n">
@@ -3422,6 +3549,11 @@
           <t>Desde 1971, site funcional porem datado; empresa grande familiar</t>
         </is>
       </c>
+      <c r="P28" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @buck_and_sons.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="n">
@@ -3493,6 +3625,11 @@
           <t>Site limpo mas datado (2022); nail bar bonito</t>
         </is>
       </c>
+      <c r="P29" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @serenitynashville.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="26" t="n">
@@ -3560,6 +3697,11 @@
           <t>Logo anos 2000, layout denso; info@ visivel</t>
         </is>
       </c>
+      <c r="P30" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @propaintingcharlotte.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="n">
@@ -3631,6 +3773,11 @@
           <t>Wix razoavel, logo fraco; IG 651</t>
         </is>
       </c>
+      <c r="P31" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @jet_exterior.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="26" t="n">
@@ -3696,6 +3843,11 @@
           <t>Desde 1957; template funcional datado-ish</t>
         </is>
       </c>
+      <c r="P32" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: e-mail do site.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="21" t="n">
@@ -3759,6 +3911,11 @@
           <t>Squarespace ok, hero com contraste ruim; desde 1945</t>
         </is>
       </c>
+      <c r="P33" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @mclainsmarketkc.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="26" t="n">
@@ -3830,6 +3987,11 @@
           <t>Template moderno ok; pouca dor aparente</t>
         </is>
       </c>
+      <c r="P34" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @squeekyscarwash.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="21" t="n">
@@ -3901,6 +4063,11 @@
           <t>Razoavel e funcional</t>
         </is>
       </c>
+      <c r="P35" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @comalfencesa.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="26" t="n">
@@ -3968,6 +4135,11 @@
           <t>Carregado mas funcional; 630 reviews; familia</t>
         </is>
       </c>
+      <c r="P36" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @functional.idaho.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="21" t="n">
@@ -4039,6 +4211,11 @@
           <t>Site razoavel com bug visual no hero; mike@ exposto</t>
         </is>
       </c>
+      <c r="P37" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @mcdaniels_landscaping.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="26" t="n">
@@ -4108,6 +4285,11 @@
           <t>Site ok generico; IG com 0 seguidores = comecando presenca social</t>
         </is>
       </c>
+      <c r="P38" s="30" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: DM em @boldwashjacksonville.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="n">
@@ -4173,6 +4355,11 @@
           <t>SUSPEITA de lead-broker: telefone placeholder 816-555-7890 na foto; verificar se e negocio real</t>
         </is>
       </c>
+      <c r="P39" s="25" t="inlineStr">
+        <is>
+          <t>Morno: so vale se sobrar tempo depois dos quentes. Canal: e-mail do site.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="26" t="n">
@@ -4236,6 +4423,11 @@
       <c r="O40" s="30" t="inlineStr">
         <is>
           <t>Moderno com social proof; desde 1976</t>
+        </is>
+      </c>
+      <c r="P40" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
         </is>
       </c>
     </row>
@@ -4295,6 +4487,11 @@
           <t>Moderno com fotos reais da equipe</t>
         </is>
       </c>
+      <c r="P41" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="26" t="n">
@@ -4362,6 +4559,11 @@
           <t>Site bom; IG com so 57 seguidores (oportunidade social, nao site)</t>
         </is>
       </c>
+      <c r="P42" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="n">
@@ -4433,6 +4635,11 @@
           <t>Site moderno bom</t>
         </is>
       </c>
+      <c r="P43" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="26" t="n">
@@ -4504,6 +4711,11 @@
           <t>Marca forte, 18+ unidades, IG 10K; provavelmente tem agencia</t>
         </is>
       </c>
+      <c r="P44" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
@@ -4571,6 +4783,11 @@
           <t>Site moderno; rede regional</t>
         </is>
       </c>
+      <c r="P45" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="26" t="n">
@@ -4642,6 +4859,11 @@
           <t>Site moderno</t>
         </is>
       </c>
+      <c r="P46" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="n">
@@ -4709,6 +4931,11 @@
           <t>Grande (4 cidades TX), video no hero</t>
         </is>
       </c>
+      <c r="P47" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="26" t="n">
@@ -4776,6 +5003,11 @@
           <t>Moderno; 10+ unidades</t>
         </is>
       </c>
+      <c r="P48" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="n">
@@ -4847,6 +5079,11 @@
           <t>Moderno, badges 2026</t>
         </is>
       </c>
+      <c r="P49" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="26" t="n">
@@ -4918,6 +5155,11 @@
           <t>Lead-gen moderno</t>
         </is>
       </c>
+      <c r="P50" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="21" t="n">
@@ -4989,6 +5231,11 @@
           <t>Moderno; franchising no menu</t>
         </is>
       </c>
+      <c r="P51" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="26" t="n">
@@ -5054,6 +5301,11 @@
           <t>Site bom com precos claros</t>
         </is>
       </c>
+      <c r="P52" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="21" t="n">
@@ -5119,6 +5371,11 @@
           <t>Moderno decente</t>
         </is>
       </c>
+      <c r="P53" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="26" t="n">
@@ -5184,6 +5441,11 @@
           <t>Site moderno bonito; hello@ exposto</t>
         </is>
       </c>
+      <c r="P54" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="n">
@@ -5249,6 +5511,11 @@
       <c r="O55" s="25" t="inlineStr">
         <is>
           <t>Site ok com badges de rating</t>
+        </is>
+      </c>
+      <c r="P55" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
         </is>
       </c>
     </row>
@@ -5312,6 +5579,11 @@
           <t>Lead-gen competente</t>
         </is>
       </c>
+      <c r="P56" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="21" t="n">
@@ -5377,6 +5649,11 @@
           <t>Site excelente</t>
         </is>
       </c>
+      <c r="P57" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="26" t="n">
@@ -5444,6 +5721,11 @@
           <t>Rede grande AZ, IG 17K</t>
         </is>
       </c>
+      <c r="P58" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="21" t="n">
@@ -5509,6 +5791,11 @@
           <t>Moderno com booking 60s</t>
         </is>
       </c>
+      <c r="P59" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="26" t="n">
@@ -5580,6 +5867,11 @@
           <t>Plataforma 80+ cidades, nao local</t>
         </is>
       </c>
+      <c r="P60" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="21" t="n">
@@ -5645,6 +5937,11 @@
           <t>Moderno bonito</t>
         </is>
       </c>
+      <c r="P61" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="26" t="n">
@@ -5706,6 +6003,11 @@
           <t>Branding forte com mascote</t>
         </is>
       </c>
+      <c r="P62" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="n">
@@ -5773,6 +6075,11 @@
           <t>Rede multi-estado, 78k reviews</t>
         </is>
       </c>
+      <c r="P63" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="n">
@@ -5838,6 +6145,11 @@
       <c r="O64" s="30" t="inlineStr">
         <is>
           <t>Squarespace minimal chique</t>
+        </is>
+      </c>
+      <c r="P64" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
         </is>
       </c>
     </row>
@@ -5897,6 +6209,11 @@
           <t>Moderno; escala nacional</t>
         </is>
       </c>
+      <c r="P65" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="26" t="n">
@@ -5964,6 +6281,11 @@
           <t>Site forte estilo HubSpot com calculadora</t>
         </is>
       </c>
+      <c r="P66" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="21" t="n">
@@ -6035,6 +6357,11 @@
           <t>Moderno forte</t>
         </is>
       </c>
+      <c r="P67" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="26" t="n">
@@ -6102,6 +6429,11 @@
           <t>Site premium chique</t>
         </is>
       </c>
+      <c r="P68" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="21" t="n">
@@ -6169,6 +6501,11 @@
           <t>Corporacao 200+ unidades</t>
         </is>
       </c>
+      <c r="P69" s="25" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="n">
@@ -6232,9 +6569,14 @@
           <t>Corporacao 75+ unidades</t>
         </is>
       </c>
+      <c r="P70" s="30" t="inlineStr">
+        <is>
+          <t>NAO abordar para venda: o site ja e bom (ou e rede grande com agencia). Use so para seguir e comentar, para entrar no grafo do nicho.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O70"/>
+  <autoFilter ref="A4:P70"/>
   <conditionalFormatting sqref="A5:A70">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>
@@ -6495,7 +6837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6507,12 +6849,13 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="58" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="74" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -6525,7 +6868,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Potencial 6+. Fluxo: seguir → comentar 2 ou 3 dias → mandar a DM com a prévia pronta.</t>
+          <t>Potencial 6+. Leia a coluna COMO ABORDAR: ela diz o canal e o gancho de cada um. Fluxo: seguir → comentar 2 ou 3 dias → mandar a DM com a prévia pronta.</t>
         </is>
       </c>
     </row>
@@ -6577,30 +6920,35 @@
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>Ângulo de abordagem</t>
+          <t>COMO ABORDAR (faça isto)</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
+          <t>O que vi no site (diagnóstico)</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>Seguiu em</t>
         </is>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr">
         <is>
           <t>Comentou em</t>
         </is>
       </c>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>DM enviada em</t>
         </is>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -6638,20 +6986,25 @@
       <c r="G5" s="22" t="inlineStr"/>
       <c r="H5" s="24" t="inlineStr"/>
       <c r="I5" s="22" t="inlineStr"/>
-      <c r="J5" s="22" t="inlineStr">
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>SEM IG e SEM e-mail no site. Ache 'Macron Mobile Detailing Columbus' no Google Maps/Facebook, ou use o formulário do próprio site. Gancho: mande a prévia junto de 'seu trabalho é premium, o site está em 2013'. Alvo nº1 da lista.</t>
+        </is>
+      </c>
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Site de 2013 com botoes bisotados; detailing premium (pacotes de USD 350) = tem caixa; redesign completo + booking</t>
         </is>
       </c>
-      <c r="K5" s="22" t="inlineStr">
+      <c r="L5" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L5" s="31" t="inlineStr"/>
-      <c r="M5" s="31" t="inlineStr"/>
-      <c r="N5" s="31" t="inlineStr"/>
-      <c r="O5" s="25" t="inlineStr"/>
+      <c r="M5" s="32" t="inlineStr"/>
+      <c r="N5" s="32" t="inlineStr"/>
+      <c r="O5" s="32" t="inlineStr"/>
+      <c r="P5" s="22" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="n">
@@ -6685,20 +7038,25 @@
       <c r="G6" s="27" t="inlineStr"/>
       <c r="H6" s="29" t="inlineStr"/>
       <c r="I6" s="27" t="inlineStr"/>
-      <c r="J6" s="27" t="inlineStr">
+      <c r="J6" s="33" t="inlineStr">
+        <is>
+          <t>SEM canal direto no site. Procure 'Octopus Car Wash' no Maps/Facebook. Gancho: print lado a lado (bolhas e clipart) contra a prévia moderna. 2 unidades familiares = fala com o dono.</t>
+        </is>
+      </c>
+      <c r="K6" s="30" t="inlineStr">
         <is>
           <t>Layout anos 2000, logo clipart, fundo de bolhas; 2 unidades familiares; redesign + booking</t>
         </is>
       </c>
-      <c r="K6" s="27" t="inlineStr">
+      <c r="L6" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L6" s="32" t="inlineStr"/>
-      <c r="M6" s="32" t="inlineStr"/>
-      <c r="N6" s="32" t="inlineStr"/>
-      <c r="O6" s="30" t="inlineStr"/>
+      <c r="M6" s="34" t="inlineStr"/>
+      <c r="N6" s="34" t="inlineStr"/>
+      <c r="O6" s="34" t="inlineStr"/>
+      <c r="P6" s="27" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="21" t="n">
@@ -6732,20 +7090,25 @@
       <c r="G7" s="22" t="inlineStr"/>
       <c r="H7" s="24" t="inlineStr"/>
       <c r="I7" s="22" t="inlineStr"/>
-      <c r="J7" s="22" t="inlineStr">
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>SEM canal direto no site. Buscar no Maps/Facebook. Gancho: 1 unidade + loja de conveniência; prévia com serviços, preços e horário bem visíveis.</t>
+        </is>
+      </c>
+      <c r="K7" s="25" t="inlineStr">
         <is>
           <t>Template generico ~2010, 1 unidade + loja de conveniencia; redesign completo</t>
         </is>
       </c>
-      <c r="K7" s="22" t="inlineStr">
+      <c r="L7" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L7" s="31" t="inlineStr"/>
-      <c r="M7" s="31" t="inlineStr"/>
-      <c r="N7" s="31" t="inlineStr"/>
-      <c r="O7" s="25" t="inlineStr"/>
+      <c r="M7" s="32" t="inlineStr"/>
+      <c r="N7" s="32" t="inlineStr"/>
+      <c r="O7" s="32" t="inlineStr"/>
+      <c r="P7" s="22" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="26" t="n">
@@ -6789,20 +7152,25 @@
           <t>info@curbsidemobiledetailing.com</t>
         </is>
       </c>
-      <c r="J8" s="27" t="inlineStr">
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>DM no @curbsidemobiledetailing (1.583) ou e-mail info@. Gancho: no ar desde 2001 é história forte que o site atual esconde; prévia destacando os 20+ anos.</t>
+        </is>
+      </c>
+      <c r="K8" s="30" t="inlineStr">
         <is>
           <t>No ar desde 2001, layout 2012, embed YouTube antigo; historia forte pra contar num site novo</t>
         </is>
       </c>
-      <c r="K8" s="27" t="inlineStr">
+      <c r="L8" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L8" s="32" t="inlineStr"/>
-      <c r="M8" s="32" t="inlineStr"/>
-      <c r="N8" s="32" t="inlineStr"/>
-      <c r="O8" s="30" t="inlineStr"/>
+      <c r="M8" s="34" t="inlineStr"/>
+      <c r="N8" s="34" t="inlineStr"/>
+      <c r="O8" s="34" t="inlineStr"/>
+      <c r="P8" s="27" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="21" t="n">
@@ -6840,20 +7208,25 @@
           <t>p.paquet@d-a-m.ca / holsej@pakskarate.com / capecoral@randori-pro.com</t>
         </is>
       </c>
-      <c r="J9" s="22" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>CUIDADO: os e-mails são de outras franquias. Ache a unidade de Orlando no Maps. Gancho: o hero da home está QUEBRADO (seção em branco com formulário solto); o print é o argumento mais fácil da lista inteira.</t>
+        </is>
+      </c>
+      <c r="K9" s="25" t="inlineStr">
         <is>
           <t>Hero quebrado (secao em branco, form solto); multi-unidades em Orlando; consertar = venda facil de mostrar</t>
         </is>
       </c>
-      <c r="K9" s="22" t="inlineStr">
+      <c r="L9" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L9" s="31" t="inlineStr"/>
-      <c r="M9" s="31" t="inlineStr"/>
-      <c r="N9" s="31" t="inlineStr"/>
-      <c r="O9" s="25" t="inlineStr"/>
+      <c r="M9" s="32" t="inlineStr"/>
+      <c r="N9" s="32" t="inlineStr"/>
+      <c r="O9" s="32" t="inlineStr"/>
+      <c r="P9" s="22" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="26" t="n">
@@ -6897,20 +7270,25 @@
           <t>contactus@purrfectgrooming.pet</t>
         </is>
       </c>
-      <c r="J10" s="27" t="inlineStr">
+      <c r="J10" s="33" t="inlineStr">
+        <is>
+          <t>DM no @purrfectgrooming.pet (4.980) ou e-mail contactus@. Gancho: hero quebrado com logo sobreposto; frota adesivada mostra que investem em marca, mas o site não acompanha. Confirme a cidade antes (parece Doral, não Orlando).</t>
+        </is>
+      </c>
+      <c r="K10" s="30" t="inlineStr">
         <is>
           <t>Hero quebrado com sobreposicao de logo; frota adesivada (investe em marca); ATENCAO: sede em Doral/Miami</t>
         </is>
       </c>
-      <c r="K10" s="27" t="inlineStr">
+      <c r="L10" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L10" s="32" t="inlineStr"/>
-      <c r="M10" s="32" t="inlineStr"/>
-      <c r="N10" s="32" t="inlineStr"/>
-      <c r="O10" s="30" t="inlineStr"/>
+      <c r="M10" s="34" t="inlineStr"/>
+      <c r="N10" s="34" t="inlineStr"/>
+      <c r="O10" s="34" t="inlineStr"/>
+      <c r="P10" s="27" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="21" t="n">
@@ -6944,20 +7322,25 @@
       <c r="G11" s="22" t="inlineStr"/>
       <c r="H11" s="24" t="inlineStr"/>
       <c r="I11" s="22" t="inlineStr"/>
-      <c r="J11" s="22" t="inlineStr">
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps/Facebook. Gancho: copyright 2011 e formulário denso; prévia com pedido de orçamento em 3 campos.</t>
+        </is>
+      </c>
+      <c r="K11" s="25" t="inlineStr">
         <is>
           <t>Copyright 2011, template bootstrap velho, form denso; negocio real com 2 telefones</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr">
+      <c r="L11" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L11" s="31" t="inlineStr"/>
-      <c r="M11" s="31" t="inlineStr"/>
-      <c r="N11" s="31" t="inlineStr"/>
-      <c r="O11" s="25" t="inlineStr"/>
+      <c r="M11" s="32" t="inlineStr"/>
+      <c r="N11" s="32" t="inlineStr"/>
+      <c r="O11" s="32" t="inlineStr"/>
+      <c r="P11" s="22" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="26" t="n">
@@ -6995,20 +7378,25 @@
           <t>mickey@phoenixautoshop.com</t>
         </is>
       </c>
-      <c r="J12" s="27" t="inlineStr">
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>E-mail DIRETO DO DONO: mickey@phoenixautoshop.com. Gancho: oficina de família desde 1979 com site Divi roxo de 2015; prévia que respeite a história e mostre agendamento.</t>
+        </is>
+      </c>
+      <c r="K12" s="30" t="inlineStr">
         <is>
           <t>Divi roxo datado ~2015; oficina familiar desde 1979; email do dono (mickey@) exposto no site</t>
         </is>
       </c>
-      <c r="K12" s="27" t="inlineStr">
+      <c r="L12" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L12" s="32" t="inlineStr"/>
-      <c r="M12" s="32" t="inlineStr"/>
-      <c r="N12" s="32" t="inlineStr"/>
-      <c r="O12" s="30" t="inlineStr"/>
+      <c r="M12" s="34" t="inlineStr"/>
+      <c r="N12" s="34" t="inlineStr"/>
+      <c r="O12" s="34" t="inlineStr"/>
+      <c r="P12" s="27" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="21" t="n">
@@ -7042,20 +7430,25 @@
       <c r="G13" s="22" t="inlineStr"/>
       <c r="H13" s="24" t="inlineStr"/>
       <c r="I13" s="22" t="inlineStr"/>
-      <c r="J13" s="22" t="inlineStr">
+      <c r="J13" s="31" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps. Gancho: visual datado com texto em Arial sobre vídeo; rede local pequena de Phoenix.</t>
+        </is>
+      </c>
+      <c r="K13" s="25" t="inlineStr">
         <is>
           <t>Visual datado, video com texto arial; rede local pequena de Phoenix</t>
         </is>
       </c>
-      <c r="K13" s="22" t="inlineStr">
+      <c r="L13" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L13" s="31" t="inlineStr"/>
-      <c r="M13" s="31" t="inlineStr"/>
-      <c r="N13" s="31" t="inlineStr"/>
-      <c r="O13" s="25" t="inlineStr"/>
+      <c r="M13" s="32" t="inlineStr"/>
+      <c r="N13" s="32" t="inlineStr"/>
+      <c r="O13" s="32" t="inlineStr"/>
+      <c r="P13" s="22" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="26" t="n">
@@ -7089,20 +7482,25 @@
       <c r="G14" s="27" t="inlineStr"/>
       <c r="H14" s="29" t="inlineStr"/>
       <c r="I14" s="27" t="inlineStr"/>
-      <c r="J14" s="27" t="inlineStr">
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>SEM canal direto. Maps/Facebook. Gancho: Weebly feito pelo próprio dono, ele já sabe que o site é fraco; prévia com galeria das cercas reais.</t>
+        </is>
+      </c>
+      <c r="K14" s="30" t="inlineStr">
         <is>
           <t>Weebly DIY, tipografia generica, fotos reais; dono fez sozinho</t>
         </is>
       </c>
-      <c r="K14" s="27" t="inlineStr">
+      <c r="L14" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L14" s="32" t="inlineStr"/>
-      <c r="M14" s="32" t="inlineStr"/>
-      <c r="N14" s="32" t="inlineStr"/>
-      <c r="O14" s="30" t="inlineStr"/>
+      <c r="M14" s="34" t="inlineStr"/>
+      <c r="N14" s="34" t="inlineStr"/>
+      <c r="O14" s="34" t="inlineStr"/>
+      <c r="P14" s="27" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="21" t="n">
@@ -7146,20 +7544,25 @@
           <t>csr@westernhvac.com / tom@westernhvac.com / max@westernhvac.com</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr">
+      <c r="J15" s="31" t="inlineStr">
+        <is>
+          <t>E-mail tom@ ou max@ (parecem os sócios) ou DM @westernhvac (2.281). Gancho: desde 1967 e Carrier dealer, mas logo 3D dos anos 2000. Empresa grande: espere decisão mais lenta.</t>
+        </is>
+      </c>
+      <c r="K15" s="25" t="inlineStr">
         <is>
           <t>Logo 3D anos 2000, botoes de ticket; desde 1967, Carrier dealer = caixa; decisao pode ser lenta</t>
         </is>
       </c>
-      <c r="K15" s="22" t="inlineStr">
+      <c r="L15" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L15" s="31" t="inlineStr"/>
-      <c r="M15" s="31" t="inlineStr"/>
-      <c r="N15" s="31" t="inlineStr"/>
-      <c r="O15" s="25" t="inlineStr"/>
+      <c r="M15" s="32" t="inlineStr"/>
+      <c r="N15" s="32" t="inlineStr"/>
+      <c r="O15" s="32" t="inlineStr"/>
+      <c r="P15" s="22" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="26" t="n">
@@ -7197,20 +7600,25 @@
           <t>info@sciotolandscaping.com</t>
         </is>
       </c>
-      <c r="J16" s="27" t="inlineStr">
+      <c r="J16" s="33" t="inlineStr">
+        <is>
+          <t>E-mail info@sciotolandscaping.com. Gancho: template de 2012 usando FOTO DE BANCO DE IMAGEM; prévia com os jardins reais que eles fizeram.</t>
+        </is>
+      </c>
+      <c r="K16" s="30" t="inlineStr">
         <is>
           <t>Template 2012 com foto de banco de imagem; info@ visivel no header</t>
         </is>
       </c>
-      <c r="K16" s="27" t="inlineStr">
+      <c r="L16" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L16" s="32" t="inlineStr"/>
-      <c r="M16" s="32" t="inlineStr"/>
-      <c r="N16" s="32" t="inlineStr"/>
-      <c r="O16" s="30" t="inlineStr"/>
+      <c r="M16" s="34" t="inlineStr"/>
+      <c r="N16" s="34" t="inlineStr"/>
+      <c r="O16" s="34" t="inlineStr"/>
+      <c r="P16" s="27" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="21" t="n">
@@ -7248,20 +7656,25 @@
           <t>straightedgepp@gmail.com</t>
         </is>
       </c>
-      <c r="J17" s="22" t="inlineStr">
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>E-mail straightedgepp@gmail.com (Gmail = negócio pequeno, o dono lê). Gancho: 49 avaliações 4.8 estrelas e o site não mostra isso em lugar nenhum.</t>
+        </is>
+      </c>
+      <c r="K17" s="25" t="inlineStr">
         <is>
           <t>Logo clipart, WP basico; 49 reviews 4.8 = negocio bom com site fraco</t>
         </is>
       </c>
-      <c r="K17" s="22" t="inlineStr">
+      <c r="L17" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L17" s="31" t="inlineStr"/>
-      <c r="M17" s="31" t="inlineStr"/>
-      <c r="N17" s="31" t="inlineStr"/>
-      <c r="O17" s="25" t="inlineStr"/>
+      <c r="M17" s="32" t="inlineStr"/>
+      <c r="N17" s="32" t="inlineStr"/>
+      <c r="O17" s="32" t="inlineStr"/>
+      <c r="P17" s="22" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="26" t="n">
@@ -7305,20 +7718,25 @@
           <t>info@allcreaturespetgrooming.com</t>
         </is>
       </c>
-      <c r="J18" s="27" t="inlineStr">
+      <c r="J18" s="33" t="inlineStr">
+        <is>
+          <t>DM no @allcreaturespetgrooming (3.277) ou e-mail info@. Gancho: Wix com logo duplicado gigante e layout desalinhado; print lado a lado resolve a conversa.</t>
+        </is>
+      </c>
+      <c r="K18" s="30" t="inlineStr">
         <is>
           <t>Wix DIY com logo duplicado gigante e layout desalinhado; tem booking</t>
         </is>
       </c>
-      <c r="K18" s="27" t="inlineStr">
+      <c r="L18" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L18" s="32" t="inlineStr"/>
-      <c r="M18" s="32" t="inlineStr"/>
-      <c r="N18" s="32" t="inlineStr"/>
-      <c r="O18" s="30" t="inlineStr"/>
+      <c r="M18" s="34" t="inlineStr"/>
+      <c r="N18" s="34" t="inlineStr"/>
+      <c r="O18" s="34" t="inlineStr"/>
+      <c r="P18" s="27" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="21" t="n">
@@ -7358,20 +7776,25 @@
         <v>4204</v>
       </c>
       <c r="I19" s="22" t="inlineStr"/>
-      <c r="J19" s="22" t="inlineStr">
+      <c r="J19" s="31" t="inlineStr">
+        <is>
+          <t>DM no @bloombakingco (4.204). SEM e-mail no site. Gancho: padaria artesanal bonita com site sem graça; prévia com as fotos dos produtos que já postam no IG.</t>
+        </is>
+      </c>
+      <c r="K19" s="25" t="inlineStr">
         <is>
           <t>Layout ~2015 (Duda), logo simples; padaria artesanal com IG</t>
         </is>
       </c>
-      <c r="K19" s="22" t="inlineStr">
+      <c r="L19" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L19" s="31" t="inlineStr"/>
-      <c r="M19" s="31" t="inlineStr"/>
-      <c r="N19" s="31" t="inlineStr"/>
-      <c r="O19" s="25" t="inlineStr"/>
+      <c r="M19" s="32" t="inlineStr"/>
+      <c r="N19" s="32" t="inlineStr"/>
+      <c r="O19" s="32" t="inlineStr"/>
+      <c r="P19" s="22" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="26" t="n">
@@ -7409,20 +7832,25 @@
           <t>bluswancarwash@gmail.com</t>
         </is>
       </c>
-      <c r="J20" s="27" t="inlineStr">
+      <c r="J20" s="33" t="inlineStr">
+        <is>
+          <t>E-mail bluswancarwash@gmail.com. Gancho: GoDaddy DIY genérico; prévia com planos e preços claros.</t>
+        </is>
+      </c>
+      <c r="K20" s="30" t="inlineStr">
         <is>
           <t>GoDaddy DIY, 1 unidade; template razoavel mas generico</t>
         </is>
       </c>
-      <c r="K20" s="27" t="inlineStr">
+      <c r="L20" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L20" s="32" t="inlineStr"/>
-      <c r="M20" s="32" t="inlineStr"/>
-      <c r="N20" s="32" t="inlineStr"/>
-      <c r="O20" s="30" t="inlineStr"/>
+      <c r="M20" s="34" t="inlineStr"/>
+      <c r="N20" s="34" t="inlineStr"/>
+      <c r="O20" s="34" t="inlineStr"/>
+      <c r="P20" s="27" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="21" t="n">
@@ -7466,20 +7894,25 @@
           <t>customerservice@alamofencesa.com</t>
         </is>
       </c>
-      <c r="J21" s="22" t="inlineStr">
+      <c r="J21" s="31" t="inlineStr">
+        <is>
+          <t>E-mail customerservice@alamofencesa.com. Gancho: layout centrado antigo. Extra: o IG tem só 88 seguidores, dá pra oferecer site + presença social.</t>
+        </is>
+      </c>
+      <c r="K21" s="25" t="inlineStr">
         <is>
           <t>Layout centrado antigo; customerservice@ exposto; negocio estabelecido</t>
         </is>
       </c>
-      <c r="K21" s="22" t="inlineStr">
+      <c r="L21" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L21" s="31" t="inlineStr"/>
-      <c r="M21" s="31" t="inlineStr"/>
-      <c r="N21" s="31" t="inlineStr"/>
-      <c r="O21" s="25" t="inlineStr"/>
+      <c r="M21" s="32" t="inlineStr"/>
+      <c r="N21" s="32" t="inlineStr"/>
+      <c r="O21" s="32" t="inlineStr"/>
+      <c r="P21" s="22" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="26" t="n">
@@ -7517,20 +7950,25 @@
           <t>service@ims365hvac.com</t>
         </is>
       </c>
-      <c r="J22" s="27" t="inlineStr">
+      <c r="J22" s="33" t="inlineStr">
+        <is>
+          <t>E-mail service@ims365hvac.com. Gancho: 25+ anos de experiência num WordPress genérico com hero cru.</t>
+        </is>
+      </c>
+      <c r="K22" s="30" t="inlineStr">
         <is>
           <t>WP generico, hero cru; empresa 25+ anos</t>
         </is>
       </c>
-      <c r="K22" s="27" t="inlineStr">
+      <c r="L22" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L22" s="32" t="inlineStr"/>
-      <c r="M22" s="32" t="inlineStr"/>
-      <c r="N22" s="32" t="inlineStr"/>
-      <c r="O22" s="30" t="inlineStr"/>
+      <c r="M22" s="34" t="inlineStr"/>
+      <c r="N22" s="34" t="inlineStr"/>
+      <c r="O22" s="34" t="inlineStr"/>
+      <c r="P22" s="27" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="21" t="n">
@@ -7574,20 +8012,25 @@
           <t>orlandoadmin@mawus.com</t>
         </is>
       </c>
-      <c r="J23" s="22" t="inlineStr">
+      <c r="J23" s="31" t="inlineStr">
+        <is>
+          <t>DM no @maworlando (1.049) ou e-mail orlandoadmin@. Gancho: logo dos anos 90; prévia com formulário de aula experimental, que é como academia capta.</t>
+        </is>
+      </c>
+      <c r="K23" s="25" t="inlineStr">
         <is>
           <t>Logo anos 90, layout mediano; academia local com programas</t>
         </is>
       </c>
-      <c r="K23" s="22" t="inlineStr">
+      <c r="L23" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L23" s="31" t="inlineStr"/>
-      <c r="M23" s="31" t="inlineStr"/>
-      <c r="N23" s="31" t="inlineStr"/>
-      <c r="O23" s="25" t="inlineStr"/>
+      <c r="M23" s="32" t="inlineStr"/>
+      <c r="N23" s="32" t="inlineStr"/>
+      <c r="O23" s="32" t="inlineStr"/>
+      <c r="P23" s="22" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="26" t="n">
@@ -7631,20 +8074,25 @@
           <t>powerwashproplus@gmail.com</t>
         </is>
       </c>
-      <c r="J24" s="27" t="inlineStr">
+      <c r="J24" s="33" t="inlineStr">
+        <is>
+          <t>E-mail powerwashproplus@gmail.com. Gancho: Squarespace genérico com logo clipart. O IG tem 7 seguidores: está começando do zero, bom candidato a site + social.</t>
+        </is>
+      </c>
+      <c r="K24" s="30" t="inlineStr">
         <is>
           <t>Squarespace generico, logo clipart, hero fraco; facil mostrar upgrade</t>
         </is>
       </c>
-      <c r="K24" s="27" t="inlineStr">
+      <c r="L24" s="27" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L24" s="32" t="inlineStr"/>
-      <c r="M24" s="32" t="inlineStr"/>
-      <c r="N24" s="32" t="inlineStr"/>
-      <c r="O24" s="30" t="inlineStr"/>
+      <c r="M24" s="34" t="inlineStr"/>
+      <c r="N24" s="34" t="inlineStr"/>
+      <c r="O24" s="34" t="inlineStr"/>
+      <c r="P24" s="27" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="21" t="n">
@@ -7688,23 +8136,28 @@
           <t>tatsbywes97@gmail.com</t>
         </is>
       </c>
-      <c r="J25" s="22" t="inlineStr">
+      <c r="J25" s="31" t="inlineStr">
+        <is>
+          <t>DM no @wes_tattoos_columbus (11K seguidores!). Gancho: artista solo desde 1997, decisão rápida e sem comitê; IG forte mas site simples, prévia com galeria destacada.</t>
+        </is>
+      </c>
+      <c r="K25" s="25" t="inlineStr">
         <is>
           <t>Artista solo desde 1997; site simples escuro; decisao rapida, IG e a vida do tatuador</t>
         </is>
       </c>
-      <c r="K25" s="22" t="inlineStr">
+      <c r="L25" s="22" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="L25" s="31" t="inlineStr"/>
-      <c r="M25" s="31" t="inlineStr"/>
-      <c r="N25" s="31" t="inlineStr"/>
-      <c r="O25" s="25" t="inlineStr"/>
+      <c r="M25" s="32" t="inlineStr"/>
+      <c r="N25" s="32" t="inlineStr"/>
+      <c r="O25" s="32" t="inlineStr"/>
+      <c r="P25" s="22" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O25"/>
+  <autoFilter ref="A4:P25"/>
   <conditionalFormatting sqref="A5:A25">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>
@@ -7714,7 +8167,7 @@
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K25">
+  <conditionalFormatting sqref="L5:L25">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
       <formula>"Ganho"</formula>
     </cfRule>
@@ -7726,7 +8179,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A fazer,Seguindo,Comentou,DM enviada,Respondeu,Prévia enviada,Negociando,Ganho,Perdido"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9287,24 +9740,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="33" t="inlineStr">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Negócio</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C4" s="35" t="inlineStr">
         <is>
           <t>O que verificar</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>Championship Martial Arts</t>
         </is>
@@ -9321,7 +9774,7 @@
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Kansas City Tree Services</t>
         </is>
@@ -9338,7 +9791,7 @@
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Purrfect Grooming</t>
         </is>
@@ -9355,7 +9808,7 @@
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>Redes grandes (nota 1-3)</t>
         </is>
@@ -9372,7 +9825,7 @@
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>E-mails genéricos</t>
         </is>

</xml_diff>